<commit_message>
Adding toolbox and monitoring objectives
</commit_message>
<xml_diff>
--- a/Monitoring Objectives Template.xlsx
+++ b/Monitoring Objectives Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25028"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25831"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\blm\dfs\loc\EGIS\ProjectsNational\AIM\Data\Development\Reports\Benchmark\Terrestrial Benchmark Tool v4.0\Monitoring Objectives Spreadsheets\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\blm.doi.net\dfs\loc\EGIS\ProjectsNational\AIM\AIMDataTools\ArcPro\Terrestrial Benchmark Tool v4.0 BETA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B2A7A27E-A628-4EF9-8E21-F1D6B21F0675}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{51A548DB-1BD3-4136-A73D-89820F21D45F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="579" xr2:uid="{BDF2D64A-487E-4672-A6D9-53FA26976B95}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="579" xr2:uid="{BDF2D64A-487E-4672-A6D9-53FA26976B95}"/>
   </bookViews>
   <sheets>
     <sheet name="Monitoring Objectives" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,11 @@
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -525,6 +529,7 @@
       <b/>
       <sz val="12"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="12"/>
@@ -532,7 +537,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -549,6 +554,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFE6E6E6"/>
         <bgColor rgb="FFE6E6E6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -668,7 +679,6 @@
   </cellStyleXfs>
   <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -704,7 +714,8 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1257,106 +1268,114 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{94F60136-2AC2-47D0-97B6-B499356FBC21}">
-  <dimension ref="A1:N32"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:N41"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="25.6328125" customWidth="1"/>
-    <col min="3" max="3" width="45.7265625" customWidth="1"/>
-    <col min="4" max="4" width="14.453125" customWidth="1"/>
-    <col min="5" max="5" width="21.81640625" customWidth="1"/>
-    <col min="6" max="6" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.5703125" customWidth="1"/>
+    <col min="3" max="3" width="45.7109375" customWidth="1"/>
+    <col min="4" max="4" width="14.42578125" customWidth="1"/>
+    <col min="5" max="5" width="21.85546875" customWidth="1"/>
+    <col min="6" max="6" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="24" customWidth="1"/>
     <col min="9" max="9" width="8" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="23" customWidth="1"/>
-    <col min="13" max="13" width="13.54296875" customWidth="1"/>
-    <col min="14" max="14" width="15.81640625" customWidth="1"/>
+    <col min="13" max="13" width="13.5703125" customWidth="1"/>
+    <col min="14" max="14" width="15.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:14" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F1" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="8" t="s">
+      <c r="G1" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="8" t="s">
+      <c r="H1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="I1" s="8" t="s">
+      <c r="I1" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="8" t="s">
+      <c r="J1" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="9" t="s">
+      <c r="K1" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="10" t="s">
+      <c r="L1" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="M1" s="11" t="s">
+      <c r="M1" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="N1" s="12" t="s">
+      <c r="N1" s="11" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="B2" s="2"/>
-      <c r="D2" s="2"/>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
       <c r="E2" s="1"/>
-      <c r="L2" s="2"/>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
       <c r="E3" s="1"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
-      <c r="J3" s="2"/>
-      <c r="K3" s="2"/>
-      <c r="L3" s="2"/>
-      <c r="M3" s="2"/>
-      <c r="N3" s="2"/>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1"/>
+      <c r="H3" s="1"/>
+      <c r="I3" s="1"/>
+      <c r="J3" s="1"/>
+      <c r="K3" s="1"/>
+      <c r="L3" s="1"/>
+      <c r="M3" s="1"/>
+      <c r="N3" s="1"/>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A4" s="1"/>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
       <c r="E4" s="1"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
-      <c r="K4" s="2"/>
-      <c r="L4" s="2"/>
-      <c r="M4" s="2"/>
-      <c r="N4" s="2"/>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="F4" s="1"/>
+      <c r="G4" s="1"/>
+      <c r="H4" s="1"/>
+      <c r="I4" s="1"/>
+      <c r="J4" s="1"/>
+      <c r="K4" s="1"/>
+      <c r="L4" s="1"/>
+      <c r="M4" s="1"/>
+      <c r="N4" s="1"/>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
@@ -1369,13 +1388,13 @@
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
-      <c r="M5" s="2"/>
-      <c r="N5" s="2"/>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="M5" s="1"/>
+      <c r="N5" s="1"/>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
       <c r="B6" s="1"/>
-      <c r="C6" s="2"/>
+      <c r="C6" s="1"/>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
       <c r="F6" s="1"/>
@@ -1385,10 +1404,10 @@
       <c r="J6" s="1"/>
       <c r="K6" s="1"/>
       <c r="L6" s="1"/>
-      <c r="M6" s="2"/>
-      <c r="N6" s="2"/>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="M6" s="1"/>
+      <c r="N6" s="1"/>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
@@ -1398,341 +1417,477 @@
       <c r="G7" s="1"/>
       <c r="H7" s="1"/>
       <c r="I7" s="1"/>
+      <c r="J7" s="1"/>
       <c r="K7" s="1"/>
       <c r="L7" s="1"/>
-      <c r="M7" s="2"/>
-      <c r="N7" s="2"/>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="M7" s="1"/>
+      <c r="N7" s="1"/>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="1"/>
       <c r="B8" s="1"/>
-      <c r="C8" s="2"/>
+      <c r="C8" s="1"/>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
       <c r="F8" s="1"/>
       <c r="G8" s="1"/>
       <c r="H8" s="1"/>
       <c r="I8" s="1"/>
+      <c r="J8" s="1"/>
       <c r="K8" s="1"/>
       <c r="L8" s="1"/>
-      <c r="M8" s="2"/>
-      <c r="N8" s="2"/>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="M8" s="1"/>
+      <c r="N8" s="1"/>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="1"/>
       <c r="B9" s="1"/>
+      <c r="C9" s="1"/>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>
       <c r="G9" s="1"/>
+      <c r="H9" s="1"/>
+      <c r="I9" s="1"/>
+      <c r="J9" s="1"/>
       <c r="K9" s="1"/>
       <c r="L9" s="1"/>
-      <c r="M9" s="2"/>
-      <c r="N9" s="2"/>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="M9" s="1"/>
+      <c r="N9" s="1"/>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" s="1"/>
       <c r="B10" s="1"/>
-      <c r="C10" s="2"/>
+      <c r="C10" s="1"/>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
       <c r="F10" s="1"/>
       <c r="G10" s="1"/>
-      <c r="H10" s="2"/>
+      <c r="H10" s="1"/>
+      <c r="I10" s="1"/>
+      <c r="J10" s="1"/>
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
-      <c r="M10" s="2"/>
-      <c r="N10" s="2"/>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="M10" s="1"/>
+      <c r="N10" s="1"/>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
-      <c r="C11" s="2"/>
+      <c r="B11" s="1"/>
+      <c r="C11" s="1"/>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>
       <c r="G11" s="1"/>
+      <c r="H11" s="1"/>
+      <c r="I11" s="1"/>
+      <c r="J11" s="1"/>
       <c r="K11" s="1"/>
       <c r="L11" s="1"/>
-      <c r="M11" s="2"/>
-      <c r="N11" s="2"/>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="M11" s="1"/>
+      <c r="N11" s="1"/>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
+      <c r="B12" s="1"/>
+      <c r="C12" s="1"/>
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
       <c r="F12" s="1"/>
       <c r="G12" s="1"/>
-      <c r="H12" s="2"/>
+      <c r="H12" s="1"/>
+      <c r="I12" s="1"/>
+      <c r="J12" s="1"/>
       <c r="K12" s="1"/>
       <c r="L12" s="1"/>
-      <c r="M12" s="2"/>
-      <c r="N12" s="2"/>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="M12" s="1"/>
+      <c r="N12" s="1"/>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="1"/>
-      <c r="C13" s="2"/>
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
+      <c r="F13" s="1"/>
       <c r="G13" s="1"/>
-      <c r="M13" s="2"/>
-      <c r="N13" s="2"/>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="H13" s="1"/>
+      <c r="I13" s="1"/>
+      <c r="J13" s="1"/>
+      <c r="K13" s="1"/>
+      <c r="L13" s="1"/>
+      <c r="M13" s="1"/>
+      <c r="N13" s="1"/>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" s="1"/>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
+      <c r="F14" s="1"/>
       <c r="G14" s="1"/>
-      <c r="M14" s="2"/>
-      <c r="N14" s="2"/>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="H14" s="1"/>
+      <c r="I14" s="1"/>
+      <c r="J14" s="1"/>
+      <c r="K14" s="1"/>
+      <c r="L14" s="1"/>
+      <c r="M14" s="1"/>
+      <c r="N14" s="1"/>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" s="1"/>
+      <c r="B15" s="1"/>
+      <c r="C15" s="1"/>
       <c r="D15" s="1"/>
       <c r="E15" s="1"/>
-      <c r="F15" s="15"/>
-      <c r="I15" s="14"/>
-      <c r="J15" s="14"/>
-      <c r="M15" s="2"/>
-      <c r="N15" s="2"/>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="F15" s="1"/>
+      <c r="G15" s="1"/>
+      <c r="H15" s="1"/>
+      <c r="I15" s="1"/>
+      <c r="J15" s="1"/>
+      <c r="K15" s="1"/>
+      <c r="L15" s="1"/>
+      <c r="M15" s="1"/>
+      <c r="N15" s="1"/>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" s="1"/>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
+      <c r="B16" s="1"/>
+      <c r="C16" s="1"/>
       <c r="D16" s="1"/>
       <c r="E16" s="1"/>
-      <c r="F16" s="15"/>
-      <c r="G16" s="2"/>
-      <c r="H16" s="2"/>
-      <c r="I16" s="14"/>
-      <c r="J16" s="14"/>
-      <c r="M16" s="2"/>
-      <c r="N16" s="2"/>
-    </row>
-    <row r="17" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="1"/>
-      <c r="D17" s="1"/>
-      <c r="E17" s="1"/>
-      <c r="F17" s="15"/>
-      <c r="I17" s="14"/>
-      <c r="J17" s="14"/>
-    </row>
-    <row r="18" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="1"/>
-      <c r="D18" s="1"/>
-      <c r="E18" s="1"/>
-      <c r="F18" s="15"/>
-      <c r="I18" s="14"/>
-      <c r="J18" s="14"/>
-    </row>
-    <row r="19" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="1"/>
-      <c r="D19" s="1"/>
-      <c r="E19" s="1"/>
-      <c r="F19" s="15"/>
-      <c r="I19" s="14"/>
-      <c r="J19" s="14"/>
-    </row>
-    <row r="20" spans="1:14" s="2" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="1"/>
-      <c r="D20" s="1"/>
-      <c r="E20" s="1"/>
-      <c r="F20" s="15"/>
-      <c r="I20" s="14"/>
-      <c r="J20" s="14"/>
-    </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="F16" s="1"/>
+      <c r="G16" s="1"/>
+      <c r="H16" s="1"/>
+      <c r="I16" s="1"/>
+      <c r="J16" s="1"/>
+      <c r="K16" s="1"/>
+      <c r="L16" s="1"/>
+      <c r="M16" s="1"/>
+      <c r="N16" s="1"/>
+    </row>
+    <row r="17" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="18" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="19" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="20" spans="1:14" s="1" customFormat="1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A21" s="1"/>
-      <c r="C21" s="2"/>
+      <c r="B21" s="1"/>
+      <c r="C21" s="1"/>
       <c r="D21" s="1"/>
       <c r="E21" s="1"/>
-      <c r="F21" s="15"/>
-      <c r="G21" s="2"/>
-      <c r="I21" s="14"/>
-      <c r="J21" s="14"/>
-      <c r="K21" s="2"/>
-      <c r="L21" s="2"/>
-      <c r="M21" s="2"/>
-      <c r="N21" s="2"/>
-    </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="F21" s="1"/>
+      <c r="G21" s="1"/>
+      <c r="H21" s="1"/>
+      <c r="I21" s="1"/>
+      <c r="J21" s="1"/>
+      <c r="K21" s="1"/>
+      <c r="L21" s="1"/>
+      <c r="M21" s="1"/>
+      <c r="N21" s="1"/>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A22" s="1"/>
-      <c r="B22" s="2"/>
-      <c r="C22" s="2"/>
+      <c r="B22" s="1"/>
+      <c r="C22" s="1"/>
       <c r="D22" s="1"/>
       <c r="E22" s="1"/>
-      <c r="F22" s="15"/>
-      <c r="G22" s="2"/>
-      <c r="H22" s="2"/>
-      <c r="I22" s="14"/>
+      <c r="F22" s="1"/>
+      <c r="G22" s="1"/>
+      <c r="H22" s="1"/>
+      <c r="I22" s="1"/>
       <c r="J22" s="14"/>
-      <c r="K22" s="2"/>
-      <c r="L22" s="2"/>
-      <c r="M22" s="2"/>
-      <c r="N22" s="2"/>
-    </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="K22" s="1"/>
+      <c r="L22" s="15"/>
+      <c r="M22" s="1"/>
+      <c r="N22" s="1"/>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>
-      <c r="B23" s="2"/>
-      <c r="C23" s="2"/>
+      <c r="B23" s="1"/>
+      <c r="C23" s="1"/>
       <c r="D23" s="1"/>
       <c r="E23" s="1"/>
-      <c r="F23" s="15"/>
-      <c r="G23" s="2"/>
-      <c r="H23" s="2"/>
-      <c r="I23" s="14"/>
+      <c r="F23" s="1"/>
+      <c r="G23" s="1"/>
+      <c r="H23" s="1"/>
+      <c r="I23" s="1"/>
       <c r="J23" s="14"/>
-      <c r="K23" s="2"/>
-      <c r="L23" s="2"/>
-      <c r="M23" s="2"/>
-      <c r="N23" s="2"/>
-    </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="K23" s="1"/>
+      <c r="L23" s="15"/>
+      <c r="M23" s="1"/>
+      <c r="N23" s="1"/>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24" s="1"/>
-      <c r="B24" s="2"/>
-      <c r="C24" s="2"/>
+      <c r="B24" s="1"/>
+      <c r="C24" s="1"/>
       <c r="D24" s="1"/>
       <c r="E24" s="1"/>
-      <c r="F24" s="15"/>
-      <c r="G24" s="2"/>
-      <c r="H24" s="2"/>
-      <c r="I24" s="14"/>
+      <c r="F24" s="1"/>
+      <c r="G24" s="1"/>
+      <c r="H24" s="1"/>
+      <c r="I24" s="1"/>
       <c r="J24" s="14"/>
-      <c r="K24" s="2"/>
-      <c r="L24" s="2"/>
-      <c r="M24" s="2"/>
-      <c r="N24" s="2"/>
-    </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="K24" s="1"/>
+      <c r="L24" s="15"/>
+      <c r="M24" s="1"/>
+      <c r="N24" s="1"/>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25" s="1"/>
-      <c r="B25" s="2"/>
-      <c r="C25" s="2"/>
+      <c r="B25" s="1"/>
+      <c r="C25" s="1"/>
       <c r="D25" s="1"/>
       <c r="E25" s="1"/>
-      <c r="F25" s="15"/>
-      <c r="G25" s="2"/>
-      <c r="H25" s="2"/>
-      <c r="I25" s="14"/>
+      <c r="F25" s="1"/>
+      <c r="G25" s="1"/>
+      <c r="H25" s="1"/>
+      <c r="I25" s="1"/>
       <c r="J25" s="14"/>
-      <c r="K25" s="2"/>
-      <c r="L25" s="2"/>
-      <c r="M25" s="2"/>
-      <c r="N25" s="2"/>
-    </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="K25" s="1"/>
+      <c r="L25" s="15"/>
+      <c r="M25" s="1"/>
+      <c r="N25" s="1"/>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26" s="1"/>
-      <c r="B26" s="2"/>
-      <c r="C26" s="2"/>
+      <c r="B26" s="1"/>
+      <c r="C26" s="1"/>
       <c r="D26" s="1"/>
       <c r="E26" s="1"/>
-      <c r="F26" s="15"/>
-      <c r="G26" s="2"/>
-      <c r="H26" s="2"/>
-      <c r="I26" s="14"/>
+      <c r="F26" s="1"/>
+      <c r="G26" s="1"/>
+      <c r="H26" s="1"/>
+      <c r="I26" s="1"/>
       <c r="J26" s="14"/>
-      <c r="K26" s="2"/>
-      <c r="L26" s="2"/>
-      <c r="M26" s="2"/>
-      <c r="N26" s="2"/>
-    </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="K26" s="1"/>
+      <c r="L26" s="15"/>
+      <c r="M26" s="1"/>
+      <c r="N26" s="1"/>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A27" s="1"/>
-      <c r="B27" s="2"/>
-      <c r="C27" s="2"/>
+      <c r="B27" s="1"/>
+      <c r="C27" s="1"/>
       <c r="D27" s="1"/>
       <c r="E27" s="1"/>
-      <c r="F27" s="15"/>
-      <c r="G27" s="2"/>
-      <c r="I27" s="14"/>
+      <c r="F27" s="1"/>
+      <c r="G27" s="1"/>
+      <c r="H27" s="1"/>
+      <c r="I27" s="1"/>
       <c r="J27" s="14"/>
-      <c r="K27" s="2"/>
-      <c r="L27" s="2"/>
-      <c r="M27" s="2"/>
-      <c r="N27" s="2"/>
-    </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="K27" s="1"/>
+      <c r="L27" s="15"/>
+      <c r="M27" s="1"/>
+      <c r="N27" s="1"/>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28" s="1"/>
-      <c r="B28" s="2"/>
-      <c r="C28" s="2"/>
+      <c r="B28" s="1"/>
+      <c r="C28" s="1"/>
       <c r="D28" s="1"/>
       <c r="E28" s="1"/>
-      <c r="F28" s="15"/>
-      <c r="G28" s="2"/>
-      <c r="H28" s="2"/>
-      <c r="I28" s="14"/>
+      <c r="F28" s="1"/>
+      <c r="G28" s="1"/>
+      <c r="H28" s="1"/>
+      <c r="I28" s="1"/>
       <c r="J28" s="14"/>
-      <c r="K28" s="2"/>
-      <c r="L28" s="2"/>
-      <c r="M28" s="2"/>
-      <c r="N28" s="2"/>
-    </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="K28" s="1"/>
+      <c r="L28" s="15"/>
+      <c r="M28" s="1"/>
+      <c r="N28" s="1"/>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A29" s="1"/>
-      <c r="B29" s="2"/>
-      <c r="C29" s="2"/>
+      <c r="B29" s="1"/>
+      <c r="C29" s="1"/>
       <c r="D29" s="1"/>
       <c r="E29" s="1"/>
-      <c r="F29" s="15"/>
-      <c r="G29" s="2"/>
-      <c r="H29" s="2"/>
-      <c r="I29" s="14"/>
+      <c r="F29" s="1"/>
+      <c r="G29" s="1"/>
+      <c r="H29" s="1"/>
+      <c r="I29" s="1"/>
       <c r="J29" s="14"/>
-      <c r="K29" s="2"/>
-      <c r="L29" s="2"/>
-      <c r="M29" s="2"/>
-      <c r="N29" s="2"/>
-    </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="K29" s="1"/>
+      <c r="L29" s="15"/>
+      <c r="M29" s="1"/>
+      <c r="N29" s="1"/>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A30" s="1"/>
-      <c r="B30" s="2"/>
-      <c r="C30" s="2"/>
+      <c r="B30" s="1"/>
+      <c r="C30" s="1"/>
       <c r="D30" s="1"/>
       <c r="E30" s="1"/>
-      <c r="F30" s="15"/>
-      <c r="G30" s="2"/>
-      <c r="H30" s="2"/>
-      <c r="I30" s="14"/>
+      <c r="F30" s="1"/>
+      <c r="G30" s="1"/>
+      <c r="H30" s="1"/>
+      <c r="I30" s="1"/>
       <c r="J30" s="14"/>
-      <c r="K30" s="2"/>
-      <c r="L30" s="2"/>
-      <c r="M30" s="2"/>
-      <c r="N30" s="2"/>
-    </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="K30" s="1"/>
+      <c r="L30" s="15"/>
+      <c r="M30" s="1"/>
+      <c r="N30" s="1"/>
+    </row>
+    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A31" s="1"/>
-      <c r="B31" s="2"/>
-      <c r="C31" s="2"/>
+      <c r="B31" s="1"/>
+      <c r="C31" s="1"/>
       <c r="D31" s="1"/>
       <c r="E31" s="1"/>
-      <c r="F31" s="15"/>
-      <c r="G31" s="2"/>
-      <c r="H31" s="2"/>
-      <c r="I31" s="14"/>
+      <c r="F31" s="1"/>
+      <c r="G31" s="1"/>
+      <c r="H31" s="1"/>
+      <c r="I31" s="1"/>
       <c r="J31" s="14"/>
-      <c r="K31" s="2"/>
-      <c r="L31" s="2"/>
-      <c r="M31" s="2"/>
-      <c r="N31" s="2"/>
-    </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="K31" s="1"/>
+      <c r="L31" s="15"/>
+      <c r="M31" s="1"/>
+      <c r="N31" s="1"/>
+    </row>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32" s="1"/>
-      <c r="B32" s="2"/>
-      <c r="C32" s="2"/>
+      <c r="B32" s="1"/>
+      <c r="C32" s="1"/>
       <c r="D32" s="1"/>
       <c r="E32" s="1"/>
-      <c r="F32" s="15"/>
-      <c r="G32" s="2"/>
-      <c r="H32" s="2"/>
-      <c r="I32" s="14"/>
+      <c r="F32" s="1"/>
+      <c r="G32" s="1"/>
+      <c r="H32" s="1"/>
+      <c r="I32" s="1"/>
       <c r="J32" s="14"/>
-      <c r="K32" s="2"/>
-      <c r="L32" s="2"/>
-      <c r="M32" s="2"/>
-      <c r="N32" s="2"/>
+      <c r="K32" s="1"/>
+      <c r="L32" s="15"/>
+      <c r="M32" s="1"/>
+      <c r="N32" s="1"/>
+    </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A33" s="1"/>
+      <c r="B33" s="1"/>
+      <c r="C33" s="1"/>
+      <c r="D33" s="1"/>
+      <c r="E33" s="1"/>
+      <c r="F33" s="1"/>
+      <c r="G33" s="1"/>
+      <c r="H33" s="1"/>
+      <c r="I33" s="1"/>
+      <c r="J33" s="14"/>
+      <c r="K33" s="1"/>
+      <c r="L33" s="15"/>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A34" s="1"/>
+      <c r="B34" s="1"/>
+      <c r="C34" s="1"/>
+      <c r="D34" s="1"/>
+      <c r="E34" s="1"/>
+      <c r="F34" s="1"/>
+      <c r="G34" s="1"/>
+      <c r="H34" s="1"/>
+      <c r="I34" s="1"/>
+      <c r="J34" s="14"/>
+      <c r="K34" s="14"/>
+      <c r="L34" s="15"/>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A35" s="1"/>
+      <c r="B35" s="1"/>
+      <c r="C35" s="1"/>
+      <c r="D35" s="1"/>
+      <c r="E35" s="1"/>
+      <c r="F35" s="1"/>
+      <c r="G35" s="1"/>
+      <c r="H35" s="1"/>
+      <c r="I35" s="1"/>
+      <c r="J35" s="14"/>
+      <c r="K35" s="14"/>
+      <c r="L35" s="15"/>
+    </row>
+    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A36" s="1"/>
+      <c r="B36" s="1"/>
+      <c r="C36" s="1"/>
+      <c r="D36" s="1"/>
+      <c r="E36" s="1"/>
+      <c r="F36" s="1"/>
+      <c r="G36" s="1"/>
+      <c r="H36" s="1"/>
+      <c r="I36" s="1"/>
+      <c r="J36" s="14"/>
+      <c r="K36" s="14"/>
+      <c r="L36" s="15"/>
+    </row>
+    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A37" s="1"/>
+      <c r="B37" s="1"/>
+      <c r="C37" s="1"/>
+      <c r="D37" s="1"/>
+      <c r="E37" s="1"/>
+      <c r="F37" s="1"/>
+      <c r="G37" s="1"/>
+      <c r="H37" s="1"/>
+      <c r="I37" s="1"/>
+      <c r="J37" s="14"/>
+      <c r="K37" s="14"/>
+      <c r="L37" s="15"/>
+    </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A38" s="1"/>
+      <c r="B38" s="1"/>
+      <c r="C38" s="1"/>
+      <c r="D38" s="1"/>
+      <c r="E38" s="1"/>
+      <c r="F38" s="1"/>
+      <c r="G38" s="1"/>
+      <c r="H38" s="1"/>
+      <c r="I38" s="1"/>
+      <c r="J38" s="14"/>
+      <c r="K38" s="14"/>
+      <c r="L38" s="15"/>
+    </row>
+    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A39" s="1"/>
+      <c r="B39" s="1"/>
+      <c r="C39" s="1"/>
+      <c r="D39" s="1"/>
+      <c r="E39" s="1"/>
+      <c r="F39" s="1"/>
+      <c r="G39" s="1"/>
+      <c r="H39" s="1"/>
+      <c r="I39" s="1"/>
+      <c r="J39" s="14"/>
+      <c r="K39" s="14"/>
+      <c r="L39" s="15"/>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A40" s="1"/>
+      <c r="B40" s="1"/>
+      <c r="C40" s="1"/>
+      <c r="D40" s="1"/>
+      <c r="E40" s="1"/>
+      <c r="F40" s="1"/>
+      <c r="G40" s="1"/>
+      <c r="H40" s="1"/>
+      <c r="I40" s="1"/>
+      <c r="J40" s="14"/>
+      <c r="K40" s="14"/>
+      <c r="L40" s="15"/>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A41" s="1"/>
+      <c r="B41" s="1"/>
+      <c r="C41" s="1"/>
+      <c r="D41" s="1"/>
+      <c r="E41" s="1"/>
+      <c r="F41" s="1"/>
+      <c r="G41" s="1"/>
+      <c r="H41" s="1"/>
+      <c r="I41" s="1"/>
+      <c r="J41" s="14"/>
+      <c r="K41" s="14"/>
+      <c r="L41" s="15"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -1741,36 +1896,24 @@
   <drawing r:id="rId2"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="5">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{8F0618DD-F646-4C04-A5F6-DBB266E109C2}">
           <x14:formula1>
             <xm:f>'Indicator Lookup'!$C$2:$C$3</xm:f>
           </x14:formula1>
-          <xm:sqref>G88:G115 I33:I173</xm:sqref>
+          <xm:sqref>G88:G115 I42:I173</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{3C5E3475-401A-4541-9453-00A1DBE3DE07}">
           <x14:formula1>
             <xm:f>'Indicator Lookup'!$D$2:$D$3</xm:f>
           </x14:formula1>
-          <xm:sqref>G33:G87</xm:sqref>
+          <xm:sqref>G42:G87</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{BECA2D09-9E7F-4EFB-B7C2-3F87786FE113}">
           <x14:formula1>
             <xm:f>'Indicator Lookup'!$A$2:$A$130</xm:f>
           </x14:formula1>
-          <xm:sqref>H2:H131</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{BE34EFE5-38C1-4CF7-9DAA-2B7738C6619B}">
-          <x14:formula1>
-            <xm:f>'Indicator Lookup'!$C$2:$C$4</xm:f>
-          </x14:formula1>
-          <xm:sqref>I2:I32</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{3F93F63E-C66E-4FC8-95AA-AA72C7DE4AE9}">
-          <x14:formula1>
-            <xm:f>'Indicator Lookup'!$D$2:$D$4</xm:f>
-          </x14:formula1>
-          <xm:sqref>G2:G32</xm:sqref>
+          <xm:sqref>H42:H131</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -1781,685 +1924,685 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E136C64-A5AE-4DD3-9E94-0A61CB935DC3}">
   <dimension ref="A1:D130"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="34.6328125" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.7265625" style="2"/>
-    <col min="3" max="4" width="10.26953125" style="2" customWidth="1"/>
-    <col min="5" max="16384" width="8.7265625" style="2"/>
+    <col min="1" max="1" width="34.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.7109375" style="1"/>
+    <col min="3" max="4" width="10.28515625" style="1" customWidth="1"/>
+    <col min="5" max="16384" width="8.7109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A1" s="13" t="s">
+    <row r="1" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="12" t="s">
         <v>146</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="13" t="s">
+    <row r="2" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A2" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="13" t="s">
+    <row r="3" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A3" s="12" t="s">
         <v>144</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A4" s="13" t="s">
+    <row r="4" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A4" s="12" t="s">
         <v>143</v>
       </c>
-      <c r="C4" s="14" t="s">
+      <c r="C4" s="13" t="s">
         <v>147</v>
       </c>
-      <c r="D4" s="14" t="s">
+      <c r="D4" s="13" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A5" s="13" t="s">
+    <row r="5" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A5" s="12" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A6" s="13" t="s">
+    <row r="6" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A6" s="12" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A7" s="13" t="s">
+    <row r="7" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A7" s="12" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A8" s="13" t="s">
+    <row r="8" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A8" s="12" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A9" s="13" t="s">
+    <row r="9" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A9" s="12" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A10" s="13" t="s">
+    <row r="10" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A10" s="12" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A11" s="13" t="s">
+    <row r="11" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A11" s="12" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A12" s="13" t="s">
+    <row r="12" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A12" s="12" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A13" s="13" t="s">
+    <row r="13" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A13" s="12" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A14" s="13" t="s">
+    <row r="14" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A14" s="12" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A15" s="13" t="s">
+    <row r="15" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A15" s="12" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A16" s="13" t="s">
+    <row r="16" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A16" s="12" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="17" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A17" s="13" t="s">
+    <row r="17" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A17" s="12" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="18" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A18" s="13" t="s">
+    <row r="18" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A18" s="12" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="19" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A19" s="13" t="s">
+    <row r="19" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A19" s="12" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="20" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A20" s="13" t="s">
+    <row r="20" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A20" s="12" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="21" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A21" s="13" t="s">
+    <row r="21" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A21" s="12" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="22" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A22" s="13" t="s">
+    <row r="22" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A22" s="12" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="23" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A23" s="13" t="s">
+    <row r="23" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A23" s="12" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="24" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A24" s="13" t="s">
+    <row r="24" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A24" s="12" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="25" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A25" s="13" t="s">
+    <row r="25" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A25" s="12" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="26" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A26" s="13" t="s">
+    <row r="26" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A26" s="12" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="27" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A27" s="13" t="s">
+    <row r="27" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A27" s="12" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="28" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A28" s="13" t="s">
+    <row r="28" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A28" s="12" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="29" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A29" s="13" t="s">
+    <row r="29" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A29" s="12" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="30" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A30" s="13" t="s">
+    <row r="30" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A30" s="12" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="31" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A31" s="13" t="s">
+    <row r="31" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A31" s="12" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="32" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A32" s="13" t="s">
+    <row r="32" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A32" s="12" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="33" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A33" s="13" t="s">
+    <row r="33" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A33" s="12" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="34" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A34" s="13" t="s">
+    <row r="34" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A34" s="12" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="35" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A35" s="13" t="s">
+    <row r="35" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A35" s="12" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="36" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A36" s="13" t="s">
+    <row r="36" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A36" s="12" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="37" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A37" s="13" t="s">
+    <row r="37" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A37" s="12" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="38" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A38" s="13" t="s">
+    <row r="38" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A38" s="12" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="39" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A39" s="13" t="s">
+    <row r="39" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A39" s="12" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="40" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A40" s="13" t="s">
+    <row r="40" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A40" s="12" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="41" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A41" s="13" t="s">
+    <row r="41" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A41" s="12" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="42" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A42" s="13" t="s">
+    <row r="42" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A42" s="12" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="43" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A43" s="13" t="s">
+    <row r="43" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A43" s="12" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="44" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A44" s="13" t="s">
+    <row r="44" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A44" s="12" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="45" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A45" s="13" t="s">
+    <row r="45" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A45" s="12" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="46" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A46" s="13" t="s">
+    <row r="46" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A46" s="12" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="47" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A47" s="13" t="s">
+    <row r="47" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A47" s="12" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="48" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A48" s="13" t="s">
+    <row r="48" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A48" s="12" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="49" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A49" s="13" t="s">
+    <row r="49" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A49" s="12" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="50" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A50" s="13" t="s">
+    <row r="50" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A50" s="12" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="51" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A51" s="13" t="s">
+    <row r="51" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A51" s="12" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="52" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A52" s="13" t="s">
+    <row r="52" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A52" s="12" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="53" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A53" s="13" t="s">
+    <row r="53" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A53" s="12" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="54" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A54" s="13" t="s">
+    <row r="54" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A54" s="12" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="55" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A55" s="13" t="s">
+    <row r="55" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A55" s="12" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="56" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A56" s="13" t="s">
+    <row r="56" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A56" s="12" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="57" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A57" s="13" t="s">
+    <row r="57" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A57" s="12" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="58" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A58" s="13" t="s">
+    <row r="58" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A58" s="12" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="59" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A59" s="13" t="s">
+    <row r="59" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A59" s="12" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="60" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A60" s="13" t="s">
+    <row r="60" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A60" s="12" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="61" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A61" s="13" t="s">
+    <row r="61" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A61" s="12" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="62" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A62" s="13" t="s">
+    <row r="62" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A62" s="12" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="63" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A63" s="13" t="s">
+    <row r="63" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A63" s="12" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="64" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A64" s="13" t="s">
+    <row r="64" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A64" s="12" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="65" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A65" s="13" t="s">
+    <row r="65" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A65" s="12" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="66" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A66" s="13" t="s">
+    <row r="66" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A66" s="12" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="67" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A67" s="13" t="s">
+    <row r="67" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A67" s="12" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="68" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A68" s="13" t="s">
+    <row r="68" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A68" s="12" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="69" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A69" s="13" t="s">
+    <row r="69" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A69" s="12" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="70" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A70" s="13" t="s">
+    <row r="70" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A70" s="12" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="71" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A71" s="13" t="s">
+    <row r="71" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A71" s="12" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="72" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A72" s="13" t="s">
+    <row r="72" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A72" s="12" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="73" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A73" s="13" t="s">
+    <row r="73" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A73" s="12" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="74" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A74" s="13" t="s">
+    <row r="74" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A74" s="12" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="75" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A75" s="13" t="s">
+    <row r="75" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A75" s="12" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="76" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A76" s="13" t="s">
+    <row r="76" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A76" s="12" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="77" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A77" s="13" t="s">
+    <row r="77" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A77" s="12" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="78" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A78" s="13" t="s">
+    <row r="78" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A78" s="12" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="79" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A79" s="13" t="s">
+    <row r="79" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A79" s="12" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="80" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A80" s="13" t="s">
+    <row r="80" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A80" s="12" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="81" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A81" s="13" t="s">
+    <row r="81" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A81" s="12" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="82" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A82" s="13" t="s">
+    <row r="82" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A82" s="12" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="83" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A83" s="13" t="s">
+    <row r="83" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A83" s="12" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="84" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A84" s="13" t="s">
+    <row r="84" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A84" s="12" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="85" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A85" s="13" t="s">
+    <row r="85" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A85" s="12" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="86" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A86" s="13" t="s">
+    <row r="86" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A86" s="12" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="87" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A87" s="13" t="s">
+    <row r="87" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A87" s="12" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="88" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A88" s="13" t="s">
+    <row r="88" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A88" s="12" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="89" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A89" s="13" t="s">
+    <row r="89" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A89" s="12" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="90" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A90" s="13" t="s">
+    <row r="90" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A90" s="12" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="91" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A91" s="13" t="s">
+    <row r="91" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A91" s="12" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="92" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A92" s="13" t="s">
+    <row r="92" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A92" s="12" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="93" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A93" s="13" t="s">
+    <row r="93" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A93" s="12" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="94" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A94" s="13" t="s">
+    <row r="94" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A94" s="12" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="95" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A95" s="13" t="s">
+    <row r="95" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A95" s="12" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="96" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A96" s="13" t="s">
+    <row r="96" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A96" s="12" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="97" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A97" s="13" t="s">
+    <row r="97" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A97" s="12" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="98" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A98" s="13" t="s">
+    <row r="98" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A98" s="12" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="99" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A99" s="13" t="s">
+    <row r="99" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A99" s="12" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="100" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A100" s="13" t="s">
+    <row r="100" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A100" s="12" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="101" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A101" s="13" t="s">
+    <row r="101" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A101" s="12" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="102" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A102" s="13" t="s">
+    <row r="102" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A102" s="12" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="103" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A103" s="13" t="s">
+    <row r="103" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A103" s="12" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="104" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A104" s="13" t="s">
+    <row r="104" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A104" s="12" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="105" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A105" s="13" t="s">
+    <row r="105" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A105" s="12" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="106" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A106" s="13" t="s">
+    <row r="106" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A106" s="12" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="107" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A107" s="13" t="s">
+    <row r="107" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A107" s="12" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="108" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A108" s="13" t="s">
+    <row r="108" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A108" s="12" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="109" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A109" s="13" t="s">
+    <row r="109" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A109" s="12" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="110" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A110" s="13" t="s">
+    <row r="110" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A110" s="12" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="111" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A111" s="13" t="s">
+    <row r="111" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A111" s="12" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="112" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A112" s="13" t="s">
+    <row r="112" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A112" s="12" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="113" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A113" s="13" t="s">
+    <row r="113" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A113" s="12" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="114" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A114" s="13" t="s">
+    <row r="114" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A114" s="12" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="115" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A115" s="13" t="s">
+    <row r="115" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A115" s="12" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="116" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A116" s="13" t="s">
+    <row r="116" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A116" s="12" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="117" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A117" s="13" t="s">
+    <row r="117" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A117" s="12" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="118" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A118" s="13" t="s">
+    <row r="118" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A118" s="12" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="119" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A119" s="13" t="s">
+    <row r="119" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A119" s="12" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="120" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A120" s="13" t="s">
+    <row r="120" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A120" s="12" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="121" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A121" s="13" t="s">
+    <row r="121" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A121" s="12" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="122" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A122" s="13" t="s">
+    <row r="122" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A122" s="12" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="123" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A123" s="13" t="s">
+    <row r="123" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A123" s="12" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="124" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A124" s="13" t="s">
+    <row r="124" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A124" s="12" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="125" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A125" s="13" t="s">
+    <row r="125" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A125" s="12" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="126" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A126" s="13" t="s">
+    <row r="126" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A126" s="12" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="127" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A127" s="13" t="s">
+    <row r="127" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A127" s="12" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="128" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A128" s="13" t="s">
+    <row r="128" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A128" s="12" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="129" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A129" s="13" t="s">
+    <row r="129" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A129" s="12" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="130" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A130" s="13" t="s">
+    <row r="130" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A130" s="12" t="s">
         <v>19</v>
       </c>
     </row>
@@ -2481,15 +2624,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010035D3E94358DD5E4094EA7A3485D29B25" ma:contentTypeVersion="5" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="42c1fa7e58f544252e42637c7e0778d3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="173833d8-5c27-4dfc-8c66-b95248c48c30" xmlns:ns4="c783a9be-6482-4e9a-a77c-ffc10e952c68" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ebb5750562a40b810f21032b63bbd02c" ns3:_="" ns4:_="">
     <xsd:import namespace="173833d8-5c27-4dfc-8c66-b95248c48c30"/>
@@ -2660,6 +2794,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7E71D8BF-7A55-427A-8985-E2F2B4BCB0F1}">
   <ds:schemaRefs>
@@ -2678,14 +2821,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6DE059C8-D763-4CB5-9FE3-1113B7F10E64}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D28F4585-C223-47F4-A327-2E922703474A}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2702,4 +2837,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6DE059C8-D763-4CB5-9FE3-1113B7F10E64}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>